<commit_message>
Add the remaining pre-send PVP findings from the client-comment and address pass.
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/L2-Step1-PVP-1400200301.01-批注清单_10-29-2026.xlsx
+++ b/L2-Step1-PVP-1400200301.01-批注清单_10-29-2026.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本版已改" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PVP 批注'!$A$1:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'本版已改'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PVP 批注'!$A$1:$F$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'本版已改'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1103,8 +1103,128 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>内部数值/逻辑</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>附录 2 第 5 项</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>PSP-140020-2026-001.01</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>标题是 Analytical Method Validation/Transfer/Verification Master Plan Protocol，编号却是 PSP-140020-2026-001.01。同表第 9 项稳定性研究才是 PSP-140020-2026-003.01。001.01 不是分析方法验证主计划的编号。外发前改成正确文件号，或改标题。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>笔误/格式</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>表 8 Sunresin 高陵生产地址</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>City Shanxi)</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>西安在陕西 Shaanxi，不是山西 Shanxi。同格 jinye 应大写为 Jinye，GaoLing 应为 Gaoling，Weiyang 的 g 不是普通英文字母，地址在 Development Zone 后多一个右括号。这是预备外发的供应商地址。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>笔误/格式</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>表 6 偶联温度，2 处</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>target: 25°C</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>表 7 目标温度是 25.0、20.0、5.0，正文大量仍是 25 °C、20 °C、5 °C。这两处写成 25°C，其中 “react at 21 - 26 (target: 25 °C)” 少了温度单位。外发前统一成一位小数，例如 25.0°C。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>笔误/格式</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>附录 2 变更条目</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>projectCPo140019</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>project 和 CPo140019 之间少空格。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F21"/>
+  <autoFilter ref="A1:F25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1116,7 +1236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1287,8 +1407,48 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Johan，2026-10-28 问 4.0 V</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>4.0 V</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>正文锚点已经是 4.0 V，整数 “4 V” 已不在。批注可关。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>附录 2 已引用 PFD</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>WI-61120</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Process Flow Document 编号 WI-61120 已列入。Johan 2026-07-22 说有了 PFD 就引用。批注可关。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>